<commit_message>
Files that hadn't been pushed into github
</commit_message>
<xml_diff>
--- a/figures/color_scheme.xlsx
+++ b/figures/color_scheme.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SynologyDrive\GITHUB\Homarine\Homarine_Catabolism_MS\figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C657888A-5958-45A9-8618-8987FF4E0CDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB7CC72A-A293-46BD-B4EE-A19BF54BFBD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{15280E9F-436A-406D-A44C-4723DF8E2193}"/>
   </bookViews>
@@ -197,9 +197,6 @@
     <t>Turquoise</t>
   </si>
   <si>
-    <t>#86C6E5</t>
-  </si>
-  <si>
     <t>Pseudomonadaceae</t>
   </si>
   <si>
@@ -216,6 +213,9 @@
   </si>
   <si>
     <t>#AEC7E8</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> #40E0D0 </t>
   </si>
 </sst>
 </file>
@@ -851,7 +851,7 @@
         <v>44</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="38.25">
@@ -859,13 +859,13 @@
         <v>27</v>
       </c>
       <c r="B18" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="25.5">
@@ -873,13 +873,13 @@
         <v>27</v>
       </c>
       <c r="B19" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="D19" s="3" t="s">
         <v>50</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>